<commit_message>
feat: concluir requisito 6 e implementar fluxo dinâmico do planeamento
</commit_message>
<xml_diff>
--- a/public/documents/requirement6/6_2/6_2_modelo_objetivos.xlsx
+++ b/public/documents/requirement6/6_2/6_2_modelo_objetivos.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiff\integra-sgi\integra-sgi\public\documents\requirement6\6_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A862A9C-DA91-47BE-BAB2-45878A38FAEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DAC4D55-67DC-40C4-8F96-C2B372019FEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Folha1" sheetId="1" r:id="rId1"/>
+    <sheet name="Objetivos" sheetId="1" r:id="rId1"/>
+    <sheet name="Legendas" sheetId="2" r:id="rId2"/>
+    <sheet name="Guia de Preenchimento" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="98">
   <si>
     <t>ID</t>
   </si>
@@ -144,13 +146,211 @@
   </si>
   <si>
     <t xml:space="preserve">AÇÕES PARA ESSE OBJETIVO </t>
+  </si>
+  <si>
+    <t>Campo</t>
+  </si>
+  <si>
+    <t>Significado</t>
+  </si>
+  <si>
+    <t>Código de identificação do objetivo (ex.: OBJ-001).</t>
+  </si>
+  <si>
+    <t>Resultado que a organização pretende alcançar.</t>
+  </si>
+  <si>
+    <t>Critério utilizado para medir o desempenho do objetivo.</t>
+  </si>
+  <si>
+    <t>Ações para esse objetivo</t>
+  </si>
+  <si>
+    <t>Principais atividades que serão realizadas para atingir o objetivo.</t>
+  </si>
+  <si>
+    <t>Recursos necessários</t>
+  </si>
+  <si>
+    <t>Recursos humanos, financeiros, tecnológicos, equipamentos ou materiais necessários.</t>
+  </si>
+  <si>
+    <t>Unidade de medida do indicador (%, kg, horas, número, m³, kWh, etc.).</t>
+  </si>
+  <si>
+    <t>Valor que se pretende atingir dentro do período definido.</t>
+  </si>
+  <si>
+    <t>Colaborador ou função responsável pelo acompanhamento do objetivo.</t>
+  </si>
+  <si>
+    <t>Monitorização Mensal</t>
+  </si>
+  <si>
+    <t>Registo periódico dos resultados obtidos em cada mês.</t>
+  </si>
+  <si>
+    <t>Resultado Esperado</t>
+  </si>
+  <si>
+    <t>Valor previsto para o indicador no final do período.</t>
+  </si>
+  <si>
+    <t>Resultado efetivamente alcançado após a consolidação dos dados.</t>
+  </si>
+  <si>
+    <t>Indica se o objetivo foi atingido ou não, de acordo com o resultado anual.</t>
+  </si>
+  <si>
+    <t>LEGENDAS</t>
+  </si>
+  <si>
+    <t>Como preencher</t>
+  </si>
+  <si>
+    <t>Exemplo</t>
+  </si>
+  <si>
+    <t>Observações</t>
+  </si>
+  <si>
+    <t>Atribua um código único para identificar o objetivo.</t>
+  </si>
+  <si>
+    <t>OBJ-001</t>
+  </si>
+  <si>
+    <t>Facilita a rastreabilidade dos objetivos.</t>
+  </si>
+  <si>
+    <t>Descreva claramente o resultado que pretende alcançar.</t>
+  </si>
+  <si>
+    <t>Reduzir o consumo de energia em 10%.</t>
+  </si>
+  <si>
+    <t>O objetivo deve ser específico, mensurável e alinhado com a política do SGI.</t>
+  </si>
+  <si>
+    <t>Defina como o desempenho será medido.</t>
+  </si>
+  <si>
+    <t>Consumo de energia (kWh).</t>
+  </si>
+  <si>
+    <t>Deve permitir acompanhar a evolução do objetivo.</t>
+  </si>
+  <si>
+    <t>Descreva as atividades necessárias para atingir a meta.</t>
+  </si>
+  <si>
+    <t>Substituir iluminação por LED; realizar formação.</t>
+  </si>
+  <si>
+    <t>Liste apenas as ações principais.</t>
+  </si>
+  <si>
+    <t>Indique os recursos necessários para implementar as ações.</t>
+  </si>
+  <si>
+    <t>Recursos financeiros, equipa técnica e equipamentos.</t>
+  </si>
+  <si>
+    <t>Inclua apenas os recursos realmente necessários.</t>
+  </si>
+  <si>
+    <t>Informe a unidade utilizada para medir o indicador.</t>
+  </si>
+  <si>
+    <t>%, Nº, kg, horas, m³, kWh.</t>
+  </si>
+  <si>
+    <t>Deve ser compatível com o indicador definido.</t>
+  </si>
+  <si>
+    <t>Defina o valor que pretende atingir.</t>
+  </si>
+  <si>
+    <t>Redução de 10%; 0 acidentes; ≤ 5 reclamações.</t>
+  </si>
+  <si>
+    <t>A meta deve ser realista e mensurável.</t>
+  </si>
+  <si>
+    <t>Indique o colaborador ou função responsável pelo acompanhamento.</t>
+  </si>
+  <si>
+    <t>Gestor Ambiental.</t>
+  </si>
+  <si>
+    <t>Preferencialmente indicar a função e não o nome da pessoa.</t>
+  </si>
+  <si>
+    <t>Registe mensalmente os resultados obtidos.</t>
+  </si>
+  <si>
+    <t>Janeiro: 1 250 kWh.</t>
+  </si>
+  <si>
+    <t>Atualize os dados durante todo o período de monitorização.</t>
+  </si>
+  <si>
+    <t>Registe o valor previsto para o final do período.</t>
+  </si>
+  <si>
+    <t>≤ 12 000 kWh/ano.</t>
+  </si>
+  <si>
+    <t>Utilizado como referência para avaliação do desempenho.</t>
+  </si>
+  <si>
+    <t>Registe o resultado consolidado do período.</t>
+  </si>
+  <si>
+    <t>11 650 kWh/ano.</t>
+  </si>
+  <si>
+    <t>Pode ser calculado automaticamente pela folha de cálculo.</t>
+  </si>
+  <si>
+    <t>Campo gerado automaticamente pela folha de cálculo.</t>
+  </si>
+  <si>
+    <t>SIM / NÃO</t>
+  </si>
+  <si>
+    <t>Indica se a meta foi atingida.</t>
+  </si>
+  <si>
+    <t>GUIA DE PREENCHIMENTO</t>
+  </si>
+  <si>
+    <t>de forma a promover a melhoria contínua do Sistema de Gestão Integrado.</t>
+  </si>
+  <si>
+    <r>
+      <t>Recomendação:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> A monitorização dos objetivos deve ser realizada periodicamente (preferencialmente todos os meses) e analisada durante as reuniões de acompanhamento e na </t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Revisão pela Gestão. Sempre que um objetivo não seja alcançado, a organização deverá avaliar as causas, implementar ações corretivas quando aplicável e rever o plano de ação ou a própria meta, </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -174,6 +374,28 @@
     <font>
       <b/>
       <sz val="32"/>
+      <color theme="0"/>
+      <name val="Cambria"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color theme="0"/>
+      <name val="Cambria"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="26"/>
       <color theme="0"/>
       <name val="Cambria"/>
       <family val="1"/>
@@ -375,7 +597,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -390,9 +612,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -405,15 +624,27 @@
     <xf numFmtId="2" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -423,6 +654,18 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -432,30 +675,23 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -485,10 +721,10 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF0F7343"/>
       <color rgb="FF203E5E"/>
       <color rgb="FF995816"/>
       <color rgb="FF980206"/>
-      <color rgb="FF0F7343"/>
       <color rgb="FFA00106"/>
       <color rgb="FF470D07"/>
     </mruColors>
@@ -548,6 +784,117 @@
         <a:xfrm>
           <a:off x="58058" y="1"/>
           <a:ext cx="921656" cy="921656"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>51662</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>28411</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>588936</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>105856</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagem 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1FFCBFD6-F6EF-4217-BD63-D639F5D2BEB6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="5623" t="10806" r="7781" b="7371"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="51662" y="28411"/>
+          <a:ext cx="635430" cy="609553"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>788488</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>41002</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagem 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{21EC4853-8C90-482E-BB0C-8EBD889B42AA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="918028" cy="932542"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -841,30 +1188,30 @@
   <sheetData>
     <row r="1" spans="2:24" ht="9" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:24" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6"/>
-      <c r="O2" s="6"/>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="6"/>
-      <c r="R2" s="6"/>
-      <c r="S2" s="6"/>
-      <c r="T2" s="6"/>
-      <c r="U2" s="6"/>
-      <c r="V2" s="6"/>
-      <c r="W2" s="6"/>
-      <c r="X2" s="6"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="27"/>
+      <c r="P2" s="27"/>
+      <c r="Q2" s="27"/>
+      <c r="R2" s="27"/>
+      <c r="S2" s="27"/>
+      <c r="T2" s="27"/>
+      <c r="U2" s="27"/>
+      <c r="V2" s="27"/>
+      <c r="W2" s="27"/>
+      <c r="X2" s="27"/>
     </row>
     <row r="4" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B4" s="5" t="s">
@@ -932,157 +1279,157 @@
       </c>
     </row>
     <row r="20" spans="2:24" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="C20" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="D20" s="12" t="s">
+      <c r="D20" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="E20" s="12" t="s">
+      <c r="E20" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="F20" s="12" t="s">
+      <c r="F20" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="G20" s="12" t="s">
+      <c r="G20" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="H20" s="13" t="s">
+      <c r="H20" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I20" s="12" t="s">
+      <c r="I20" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="J20" s="14" t="s">
+      <c r="J20" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="K20" s="15"/>
-      <c r="L20" s="15"/>
-      <c r="M20" s="15"/>
-      <c r="N20" s="15"/>
-      <c r="O20" s="15"/>
-      <c r="P20" s="15"/>
-      <c r="Q20" s="15"/>
-      <c r="R20" s="15"/>
-      <c r="S20" s="15"/>
-      <c r="T20" s="15"/>
-      <c r="U20" s="16"/>
-      <c r="V20" s="17" t="s">
+      <c r="K20" s="18"/>
+      <c r="L20" s="18"/>
+      <c r="M20" s="18"/>
+      <c r="N20" s="18"/>
+      <c r="O20" s="18"/>
+      <c r="P20" s="18"/>
+      <c r="Q20" s="18"/>
+      <c r="R20" s="18"/>
+      <c r="S20" s="18"/>
+      <c r="T20" s="18"/>
+      <c r="U20" s="19"/>
+      <c r="V20" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="W20" s="18"/>
-      <c r="X20" s="19"/>
+      <c r="W20" s="25"/>
+      <c r="X20" s="26"/>
     </row>
     <row r="21" spans="2:24" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="B21" s="20"/>
-      <c r="C21" s="21"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
-      <c r="G21" s="21"/>
-      <c r="H21" s="22"/>
-      <c r="I21" s="21"/>
-      <c r="J21" s="23" t="s">
+      <c r="B21" s="21"/>
+      <c r="C21" s="23"/>
+      <c r="D21" s="23"/>
+      <c r="E21" s="23"/>
+      <c r="F21" s="23"/>
+      <c r="G21" s="23"/>
+      <c r="H21" s="16"/>
+      <c r="I21" s="23"/>
+      <c r="J21" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="K21" s="23" t="s">
+      <c r="K21" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="L21" s="23" t="s">
+      <c r="L21" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="M21" s="23" t="s">
+      <c r="M21" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="N21" s="23" t="s">
+      <c r="N21" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="O21" s="23" t="s">
+      <c r="O21" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="P21" s="23" t="s">
+      <c r="P21" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="Q21" s="23" t="s">
+      <c r="Q21" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="R21" s="24" t="s">
+      <c r="R21" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="S21" s="25" t="s">
+      <c r="S21" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="T21" s="23" t="s">
+      <c r="T21" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="U21" s="23" t="s">
+      <c r="U21" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="V21" s="23" t="s">
+      <c r="V21" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="W21" s="26" t="s">
+      <c r="W21" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="X21" s="27" t="s">
+      <c r="X21" s="14" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="22" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="B22" s="8"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
-      <c r="H22" s="8"/>
-      <c r="I22" s="8"/>
-      <c r="J22" s="8"/>
-      <c r="K22" s="8"/>
-      <c r="L22" s="8"/>
-      <c r="M22" s="8"/>
-      <c r="N22" s="8"/>
-      <c r="O22" s="8"/>
-      <c r="P22" s="8"/>
-      <c r="Q22" s="8"/>
-      <c r="R22" s="8"/>
-      <c r="S22" s="8"/>
-      <c r="T22" s="8"/>
-      <c r="U22" s="8"/>
-      <c r="V22" s="8"/>
-      <c r="W22" s="10"/>
-      <c r="X22" s="9" t="str">
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="7"/>
+      <c r="J22" s="7"/>
+      <c r="K22" s="7"/>
+      <c r="L22" s="7"/>
+      <c r="M22" s="7"/>
+      <c r="N22" s="7"/>
+      <c r="O22" s="7"/>
+      <c r="P22" s="7"/>
+      <c r="Q22" s="7"/>
+      <c r="R22" s="7"/>
+      <c r="S22" s="7"/>
+      <c r="T22" s="7"/>
+      <c r="U22" s="7"/>
+      <c r="V22" s="7"/>
+      <c r="W22" s="9"/>
+      <c r="X22" s="8" t="str">
         <f>IF(W22&lt;V22, "SIM","NÃO")</f>
         <v>NÃO</v>
       </c>
     </row>
     <row r="23" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="7"/>
-      <c r="H23" s="7"/>
-      <c r="I23" s="7"/>
-      <c r="J23" s="7"/>
-      <c r="K23" s="7"/>
-      <c r="L23" s="7"/>
-      <c r="M23" s="7"/>
-      <c r="N23" s="7"/>
-      <c r="O23" s="7"/>
-      <c r="P23" s="7"/>
-      <c r="Q23" s="7"/>
-      <c r="R23" s="7"/>
-      <c r="S23" s="7"/>
-      <c r="T23" s="7"/>
-      <c r="U23" s="7"/>
-      <c r="V23" s="7"/>
-      <c r="W23" s="7"/>
-      <c r="X23" s="7" t="str">
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="6"/>
+      <c r="K23" s="6"/>
+      <c r="L23" s="6"/>
+      <c r="M23" s="6"/>
+      <c r="N23" s="6"/>
+      <c r="O23" s="6"/>
+      <c r="P23" s="6"/>
+      <c r="Q23" s="6"/>
+      <c r="R23" s="6"/>
+      <c r="S23" s="6"/>
+      <c r="T23" s="6"/>
+      <c r="U23" s="6"/>
+      <c r="V23" s="6"/>
+      <c r="W23" s="6"/>
+      <c r="X23" s="6" t="str">
         <f>IF(W23&lt;V23, "SIM","NÃO")</f>
         <v>NÃO</v>
       </c>
@@ -1117,6 +1464,9 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="V20:X20"/>
+    <mergeCell ref="C2:X2"/>
+    <mergeCell ref="E20:E21"/>
     <mergeCell ref="H20:H21"/>
     <mergeCell ref="J20:U20"/>
     <mergeCell ref="B20:B21"/>
@@ -1125,9 +1475,6 @@
     <mergeCell ref="G20:G21"/>
     <mergeCell ref="I20:I21"/>
     <mergeCell ref="F20:F21"/>
-    <mergeCell ref="V20:X20"/>
-    <mergeCell ref="C2:X2"/>
-    <mergeCell ref="E20:E21"/>
   </mergeCells>
   <conditionalFormatting sqref="X22:X24">
     <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="SIM">
@@ -1140,4 +1487,363 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8128DE40-9698-4D30-9D73-4E8E876D49A7}">
+  <dimension ref="B1:C16"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="1.44140625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="21.44140625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="55.6640625" style="5" customWidth="1"/>
+    <col min="4" max="16384" width="8.88671875" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:3" ht="6.6" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:3" ht="35.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="30" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" s="30"/>
+    </row>
+    <row r="4" spans="2:3" ht="19.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="29" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="29" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="29" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="29" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="29" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="29" t="s">
+        <v>48</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="29" t="s">
+        <v>50</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="29" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="16" spans="2:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52615416-180C-477A-81B6-A63CF98F1B29}">
+  <dimension ref="B1:E20"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="1.88671875" style="28" customWidth="1"/>
+    <col min="2" max="2" width="20.109375" style="28" customWidth="1"/>
+    <col min="3" max="3" width="38.109375" style="28" customWidth="1"/>
+    <col min="4" max="4" width="32.21875" style="28" customWidth="1"/>
+    <col min="5" max="5" width="31.109375" style="28" customWidth="1"/>
+    <col min="6" max="16384" width="8.88671875" style="28"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:5" ht="8.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:5" ht="61.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="31" t="s">
+        <v>94</v>
+      </c>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+    </row>
+    <row r="4" spans="2:5" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B4" s="32" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B5" s="33" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B6" s="33" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="29" t="s">
+        <v>55</v>
+      </c>
+      <c r="D8" s="29" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" s="29" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="29" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="29" t="s">
+        <v>2</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="29" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="29" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="29" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="29" t="s">
+        <v>48</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="29" t="s">
+        <v>50</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="29" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:E2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>